<commit_message>
The commit as used in the paper; add README, LICENCE
</commit_message>
<xml_diff>
--- a/input/phages.xlsx
+++ b/input/phages.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="0" windowWidth="16080" windowHeight="7780"/>
+    <workbookView activeTab="0" windowWidth="16140" windowHeight="7720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44" count="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43" count="43">
   <si>
     <t>Isolate</t>
   </si>
@@ -142,9 +142,6 @@
   </si>
   <si>
     <t>D</t>
-  </si>
-  <si>
-    <t>Ga0063588_100037_PP</t>
   </si>
   <si>
     <t>F</t>
@@ -219,23 +216,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <dimension ref="A1:XFD50"/>
+  <sheetFormatPr defaultColWidth="67.5" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" style="0" width="9.142307692307693"/>
+    <col min="1" max="1" style="0" width="9.142307692307693" bestFit="1" customWidth="1"/>
     <col min="2" max="2" style="0" width="16.141887019230772" customWidth="1"/>
     <col min="3" max="3" style="0" width="13.284915865384617" bestFit="1" customWidth="1"/>
     <col min="4" max="4" style="0" width="13.284915865384617" customWidth="1"/>
-    <col min="5" max="6" style="0" width="9.142307692307693"/>
+    <col min="5" max="6" style="0" width="9.142307692307693" bestFit="1" customWidth="1"/>
     <col min="7" max="7" style="0" width="12.142127403846155" bestFit="1" customWidth="1"/>
     <col min="8" max="8" style="0" width="11.28503605769231" customWidth="1"/>
     <col min="9" max="9" style="0" width="22.141526442307693" bestFit="1" customWidth="1"/>
     <col min="10" max="10" style="0" width="29.85534855769231" bestFit="1" customWidth="1"/>
     <col min="11" max="11" style="0" width="53.56820913461539" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" style="0" width="9.142307692307693"/>
+    <col min="12" max="16384" style="0" width="9.142307692307693" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="13.5">
+    <row r="1" spans="1:16384" ht="13.5">
       <c r="B1" t="inlineStr">
         <is>
           <t>Phage</t>
@@ -302,7 +299,7 @@
         </is>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="13.5">
+    <row r="2" spans="1:16384" ht="13.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -352,7 +349,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="13.5">
+    <row r="3" spans="1:16384" ht="13.5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -403,7 +400,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="13.5">
+    <row r="4" spans="1:16384" ht="13.5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -445,7 +442,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="13.5">
+    <row r="5" spans="1:16384" ht="13.5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -489,7 +486,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="13.5">
+    <row r="6" spans="1:16384" ht="13.5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -537,7 +534,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="13.5">
+    <row r="7" spans="1:16384" ht="13.5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -570,7 +567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="13.5">
+    <row r="8" spans="1:16384" ht="13.5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -623,7 +620,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="13.5">
+    <row r="9" spans="1:16384" ht="13.5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -667,7 +664,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="13.5">
+    <row r="10" spans="1:16384" ht="13.5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -702,7 +699,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="13.5">
+    <row r="11" spans="1:16384" ht="13.5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -751,7 +748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="13.5">
+    <row r="12" spans="1:16384" ht="13.5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -793,7 +790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="13.5">
+    <row r="13" spans="1:16384" ht="13.5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -844,7 +841,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="13.5">
+    <row r="14" spans="1:16384" ht="13.5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -886,7 +883,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="13.5">
+    <row r="15" spans="1:16384" ht="13.5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -928,7 +925,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="13.5">
+    <row r="16" spans="1:16384" ht="13.5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -977,7 +974,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="13.5">
+    <row r="17" spans="1:16384" ht="13.5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1019,7 +1016,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="13.5">
+    <row r="18" spans="1:16384" ht="13.5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1061,7 +1058,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="13.5">
+    <row r="19" spans="1:16384" ht="13.5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1105,7 +1102,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="13.5">
+    <row r="20" spans="1:16384" ht="13.5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1149,7 +1146,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="13.5">
+    <row r="21" spans="1:16384" ht="13.5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1184,7 +1181,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="13.5">
+    <row r="22" spans="1:16384" ht="13.5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1221,7 +1218,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="13.5">
+    <row r="23" spans="1:16384" ht="13.5">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1267,7 +1264,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="13.5">
+    <row r="24" spans="1:16384" ht="15">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1312,7 +1309,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="13.5">
+    <row r="25" spans="1:16384" ht="13.5">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1362,7 +1359,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="13.5">
+    <row r="26" spans="1:16384" ht="13.5">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1408,7 +1405,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="13.5">
+    <row r="27" spans="1:16384" ht="13.5">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1452,7 +1449,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="13.5">
+    <row r="28" spans="1:16384" ht="13.5">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1494,7 +1491,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="13.5">
+    <row r="29" spans="1:16384" ht="13.5">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1536,7 +1533,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="13.5">
+    <row r="30" spans="1:16384" ht="13.5">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1578,7 +1575,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="13.5">
+    <row r="31" spans="1:16384" ht="13.5">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1623,7 +1620,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="13.5">
+    <row r="32" spans="1:16384" ht="13.5">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1665,7 +1662,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="13.5">
+    <row r="33" spans="1:16384" ht="13.5">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1707,7 +1704,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="13.5">
+    <row r="34" spans="1:16384" ht="13.5">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1753,7 +1750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="13.5">
+    <row r="35" spans="1:16384" ht="13.5">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1788,12 +1785,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="13.5">
+    <row r="36" spans="1:16384" ht="13.5">
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36" t="s">
-        <v>39</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ga0063588_100037_PP</t>
+        </is>
       </c>
       <c r="C36" t="s">
         <v>18</v>
@@ -1841,7 +1840,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="13.5">
+    <row r="37" spans="1:16384" ht="13.5">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1862,7 +1861,7 @@
         <v>1</v>
       </c>
       <c r="G37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J37" t="s">
         <v>16</v>
@@ -1874,7 +1873,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="13.5">
+    <row r="38" spans="1:16384" ht="13.5">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1895,7 +1894,7 @@
         <v>1</v>
       </c>
       <c r="G38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -1921,7 +1920,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="13.5">
+    <row r="39" spans="1:16384" ht="13.5">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1939,16 +1938,16 @@
         </is>
       </c>
       <c r="F39" t="s">
+        <v>40</v>
+      </c>
+      <c r="H39" t="s">
         <v>41</v>
       </c>
-      <c r="H39" t="s">
+      <c r="K39" t="s">
         <v>42</v>
       </c>
-      <c r="K39" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="13.5">
+    </row>
+    <row r="40" spans="1:16384" ht="13.5">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1966,16 +1965,16 @@
         </is>
       </c>
       <c r="F40" t="s">
+        <v>40</v>
+      </c>
+      <c r="H40" t="s">
         <v>41</v>
       </c>
-      <c r="H40" t="s">
+      <c r="K40" t="s">
         <v>42</v>
       </c>
-      <c r="K40" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="13.5">
+    </row>
+    <row r="41" spans="1:16384" ht="13.5">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1993,7 +1992,7 @@
         </is>
       </c>
       <c r="F41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2006,15 +2005,15 @@
         </is>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="13.5"/>
-    <row r="43" spans="1:14" ht="13.5"/>
-    <row r="44" spans="1:14" ht="13.5"/>
-    <row r="45" spans="1:14" ht="13.5"/>
-    <row r="46" spans="1:14" ht="13.5"/>
-    <row r="47" spans="1:14" ht="13.5"/>
-    <row r="48" spans="1:14" ht="13.5"/>
-    <row r="49" spans="1:14" ht="13.5"/>
-    <row r="50" spans="1:14" ht="13.5"/>
+    <row r="42" spans="1:16384" ht="13.5"/>
+    <row r="43" spans="1:16384" ht="13.5"/>
+    <row r="44" spans="1:16384" ht="13.5"/>
+    <row r="45" spans="1:16384" ht="13.5"/>
+    <row r="46" spans="1:16384" ht="13.5"/>
+    <row r="47" spans="1:16384" ht="13.5"/>
+    <row r="48" spans="1:16384" ht="13.5"/>
+    <row r="49" spans="1:16384" ht="13.5"/>
+    <row r="50" spans="1:16384" ht="13.5"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
   <printOptions/>
@@ -2032,10 +2031,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <dimension ref="A1:XFD1"/>
+  <sheetFormatPr defaultColWidth="67.5" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="16384" style="0" width="9.142307692307693"/>
+    <col min="1" max="16384" style="0" width="9.142307692307693" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData/>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -2054,10 +2053,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <dimension ref="A1:XFD1"/>
+  <sheetFormatPr defaultColWidth="67.5" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="16384" style="0" width="9.142307692307693"/>
+    <col min="1" max="16384" style="0" width="9.142307692307693" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData/>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>

</xml_diff>